<commit_message>
update person cards and better score calculation
</commit_message>
<xml_diff>
--- a/sample.xlsx
+++ b/sample.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gille\Documents\GroepsleidingTool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{496D0953-1A5B-4C48-B5FC-928ECACAAF6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6DE250D-AD89-45E0-8BA1-E3A9731F75B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{68B1BAB8-63FB-4B81-AAF6-6A1FFD5A6052}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="17">
   <si>
     <t>Naam</t>
   </si>
@@ -37,21 +37,6 @@
     <t>Gilles</t>
   </si>
   <si>
-    <t>Welpen</t>
-  </si>
-  <si>
-    <t>Pioniers</t>
-  </si>
-  <si>
-    <t>Scouts</t>
-  </si>
-  <si>
-    <t>Erik</t>
-  </si>
-  <si>
-    <t>Tom</t>
-  </si>
-  <si>
     <t>TuurW</t>
   </si>
   <si>
@@ -62,6 +47,30 @@
   </si>
   <si>
     <t>Tak3</t>
+  </si>
+  <si>
+    <t>Jelle</t>
+  </si>
+  <si>
+    <t>Givers</t>
+  </si>
+  <si>
+    <t>Wouters</t>
+  </si>
+  <si>
+    <t>Jonggivers</t>
+  </si>
+  <si>
+    <t>Kapoenen</t>
+  </si>
+  <si>
+    <t>Obe</t>
+  </si>
+  <si>
+    <t>Bunker</t>
+  </si>
+  <si>
+    <t>Bunker,Gilles</t>
   </si>
 </sst>
 </file>
@@ -922,7 +931,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18BC5BB0-5D58-4E15-A2F3-00A2F16DB7A3}">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
@@ -930,13 +939,13 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="C1" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="D1" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E1" t="s">
         <v>1</v>
@@ -953,19 +962,19 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F2" t="s">
         <v>5</v>
-      </c>
-      <c r="C2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F2" t="s">
-        <v>9</v>
       </c>
       <c r="G2">
         <v>3</v>
@@ -973,25 +982,94 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" t="s">
         <v>10</v>
       </c>
-      <c r="B3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" t="s">
-        <v>5</v>
-      </c>
       <c r="D3" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="E3" t="s">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="F3" t="s">
         <v>4</v>
       </c>
       <c r="G3">
         <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6" t="s">
+        <v>5</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+      <c r="G6">
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
men/women count per tak and rijbewijs count
</commit_message>
<xml_diff>
--- a/sample.xlsx
+++ b/sample.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gille\Documents\GroepsleidingTool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6DE250D-AD89-45E0-8BA1-E3A9731F75B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE41EC30-F627-4A96-BD46-42A889F75CD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{68B1BAB8-63FB-4B81-AAF6-6A1FFD5A6052}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="22">
   <si>
     <t>Naam</t>
   </si>
@@ -71,6 +71,21 @@
   </si>
   <si>
     <t>Bunker,Gilles</t>
+  </si>
+  <si>
+    <t>Geslacht</t>
+  </si>
+  <si>
+    <t>M</t>
+  </si>
+  <si>
+    <t>Rijbewijs</t>
+  </si>
+  <si>
+    <t>Ja</t>
+  </si>
+  <si>
+    <t>Nee</t>
   </si>
 </sst>
 </file>
@@ -931,10 +946,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18BC5BB0-5D58-4E15-A2F3-00A2F16DB7A3}">
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -956,8 +971,14 @@
       <c r="G1" t="s">
         <v>3</v>
       </c>
+      <c r="H1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I1" t="s">
+        <v>19</v>
+      </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -979,8 +1000,14 @@
       <c r="G2">
         <v>3</v>
       </c>
+      <c r="H2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I2" t="s">
+        <v>20</v>
+      </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -1002,8 +1029,14 @@
       <c r="G3">
         <v>8</v>
       </c>
+      <c r="H3" t="s">
+        <v>18</v>
+      </c>
+      <c r="I3" t="s">
+        <v>20</v>
+      </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1025,8 +1058,14 @@
       <c r="G4">
         <v>10</v>
       </c>
+      <c r="H4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I4" t="s">
+        <v>21</v>
+      </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>15</v>
       </c>
@@ -1048,8 +1087,14 @@
       <c r="G5">
         <v>5</v>
       </c>
+      <c r="H5" t="s">
+        <v>18</v>
+      </c>
+      <c r="I5" t="s">
+        <v>21</v>
+      </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -1070,6 +1115,12 @@
       </c>
       <c r="G6">
         <v>7</v>
+      </c>
+      <c r="H6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I6" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
gender color when unassigned
</commit_message>
<xml_diff>
--- a/sample.xlsx
+++ b/sample.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gille\Documents\GroepsleidingTool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F279D81-C6EF-405D-A84C-96164E11E2A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{012258BB-E1D5-4BF6-9248-EFECAE7878D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{68B1BAB8-63FB-4B81-AAF6-6A1FFD5A6052}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="26">
   <si>
     <t>Naam</t>
   </si>
@@ -34,12 +34,6 @@
     <t>prioriteit</t>
   </si>
   <si>
-    <t>Gilles</t>
-  </si>
-  <si>
-    <t>TuurW</t>
-  </si>
-  <si>
     <t>Tak1</t>
   </si>
   <si>
@@ -49,9 +43,6 @@
     <t>Tak3</t>
   </si>
   <si>
-    <t>Jelle</t>
-  </si>
-  <si>
     <t>Givers</t>
   </si>
   <si>
@@ -64,15 +55,6 @@
     <t>Kapoenen</t>
   </si>
   <si>
-    <t>Obe</t>
-  </si>
-  <si>
-    <t>Bunker</t>
-  </si>
-  <si>
-    <t>Bunker,Gilles</t>
-  </si>
-  <si>
     <t>Geslacht</t>
   </si>
   <si>
@@ -89,6 +71,33 @@
   </si>
   <si>
     <t>Ervaring</t>
+  </si>
+  <si>
+    <t>V</t>
+  </si>
+  <si>
+    <t>Thomas</t>
+  </si>
+  <si>
+    <t>Jarne,Thomas</t>
+  </si>
+  <si>
+    <t>Jarne</t>
+  </si>
+  <si>
+    <t>Arno</t>
+  </si>
+  <si>
+    <t>Tibo</t>
+  </si>
+  <si>
+    <t>Simon</t>
+  </si>
+  <si>
+    <t>Eline</t>
+  </si>
+  <si>
+    <t>Thomas,Simon</t>
   </si>
 </sst>
 </file>
@@ -949,7 +958,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18BC5BB0-5D58-4E15-A2F3-00A2F16DB7A3}">
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
@@ -957,13 +966,13 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" t="s">
         <v>6</v>
-      </c>
-      <c r="C1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D1" t="s">
-        <v>8</v>
       </c>
       <c r="E1" t="s">
         <v>1</v>
@@ -975,42 +984,42 @@
         <v>3</v>
       </c>
       <c r="H1" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="I1" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="J1" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="B2" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D2" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E2" t="s">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="F2" t="s">
-        <v>5</v>
+        <v>23</v>
       </c>
       <c r="G2">
         <v>3</v>
       </c>
       <c r="H2" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="I2" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="J2">
         <v>2</v>
@@ -1018,31 +1027,31 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>5</v>
+        <v>23</v>
       </c>
       <c r="B3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C3" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D3" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E3" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="F3" t="s">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="G3">
         <v>8</v>
       </c>
       <c r="H3" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="I3" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="J3">
         <v>3</v>
@@ -1050,31 +1059,31 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" t="s">
         <v>9</v>
       </c>
-      <c r="B4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" t="s">
-        <v>10</v>
-      </c>
-      <c r="D4" t="s">
-        <v>12</v>
-      </c>
       <c r="E4" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="F4" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="G4">
         <v>10</v>
       </c>
       <c r="H4" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="I4" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="J4">
         <v>4</v>
@@ -1082,31 +1091,31 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="B5" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C5" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D5" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E5" t="s">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="F5" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="G5">
         <v>5</v>
       </c>
       <c r="H5" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="I5" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="J5">
         <v>7</v>
@@ -1114,34 +1123,66 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="B6" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D6" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E6" t="s">
-        <v>5</v>
+        <v>23</v>
       </c>
       <c r="F6" t="s">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="G6">
         <v>7</v>
       </c>
       <c r="H6" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="I6" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="J6">
         <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E7" t="s">
+        <v>23</v>
+      </c>
+      <c r="F7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G7">
+        <v>2</v>
+      </c>
+      <c r="H7" t="s">
+        <v>17</v>
+      </c>
+      <c r="I7" t="s">
+        <v>15</v>
+      </c>
+      <c r="J7">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>